<commit_message>
F2026 calendar: encode all 2026-08-17 decisions
- Review day -> cylindrical/spherical coordinate-systems day (5.5, 5.7)
- Feynman Vol II Ch 2-3 assigned BEFORE Felder 8.6-8.7 (geometric
  definitions of div/curl first); Ch 3 also cited on the theorems day
- Fourier series compressed to 2 days (9.1-9.3, 9.4-9.5)
- PDEs protected with 2 days (11.1-11.2+11.4, then 11.3)
- Fourier transforms (9.6) ride the Dec 14 finale, taught graphically
- 2.6-2.7 convergence cut with Appendix C pointer on the Taylor day
- Non-Newtonian Scientist due mid-semester, Mon Oct 26 (EXTRA_DUE)
- README + TODO updated (decisions locked; PCCIs Gary's way; next big
  task = re-cut WHWs to the new calendar + per-day PCCI assignments)

Regenerated PHY210 F2026 Calendar.xlsx; 39-slot and 1000-point asserts
pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -889,10 +889,14 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Practice / review day</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>5.5, 5.7; App. D</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>WHW10</t>
@@ -1093,12 +1097,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Gradient, divergence, curl</t>
+          <t>Divergence and curl, geometrically</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>8.5-8.7</t>
+          <t>Feynman Vol II Ch 2-3</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr"/>
@@ -1266,7 +1270,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10</t>
+          <t>8.9-8.10; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr"/>
@@ -1395,7 +1399,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5</t>
+          <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
@@ -1413,12 +1417,12 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains</t>
+          <t>Fourier series: different periods, finite domains, complex exponentials</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.4-9.5</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr"/>
@@ -1461,12 +1465,12 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Fourier series with complex exponentials</t>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>11.1-11.2, 11.4</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -1517,12 +1521,12 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation</t>
+          <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2</t>
+          <t>11.3, 9.6</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr"/>
@@ -1550,7 +1554,11 @@
           <t>6.3-6.4</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr"/>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>

</xml_diff>

<commit_message>
F2026 calendar: PCCI column + WHW Problem Lists tab
PCCIs (Gary-Felder style, decided 2026-08-17): 35 assignments, one per
non-quiz/non-flex class day, inline on the Schedule tab -- mostly the
day's Discovery Exercise, every number attested in a predecessor's
actual assignment (Gary's PCCI schedules, Gillian's WHW forms, Casey's
in-class sets). New 'WHW Problem Lists' tab: 13 weekly tiered lists
(Warm-up/Essentials/Depth) re-cut from Gillian's transcribed S26 forms
onto the F2026 week boundaries, with attested supplements for the
units S26 lacked (coordinates day, Feynman/8.x days, Ch 10 split);
Gillian's standing preamble at the top for Moodle copy-paste. Asserts:
PCCIs only on class days, never quiz days; WHW tab numbers match the
calendar's 13 Friday WHWs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -79,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -89,6 +90,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -457,23 +461,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,45 +510,55 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>HW Due</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Exams</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Topics</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Reading Due</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>HW Due</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Exams</t>
         </is>
@@ -570,35 +586,45 @@
           <t>1.1-1.2</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="n">
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="n">
+      <c r="K2" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Fri Oct 30</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Finding eigenvalues and eigenvectors</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.8.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>WHW08</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -624,33 +650,43 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>DE 1.2.1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>WHW01</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="n">
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="K3" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 2</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Eigenvalues and eigenvectors, continued</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>6.8</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>6.166</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -674,31 +710,41 @@
           <t>1.3</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.3.1 Part 1</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="n">
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J4" s="2" t="n">
+      <c r="K4" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 4</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>The two-coupled-oscillator problem</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>6.9</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
-      <c r="O4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>6.175</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -722,35 +768,45 @@
           <t>1.5</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.5.1 Parts 1-5</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="n">
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="J5" s="2" t="n">
+      <c r="K5" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 6</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>5.1-5.2</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -776,33 +832,43 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>DE 1.6.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
           <t>WHW02</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="n">
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="2" t="n">
+      <c r="K6" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 9</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>Cartesian 2D integrals; polar coordinates</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>5.3-5.4, 5.6</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr"/>
-      <c r="O6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.4.1</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -826,31 +892,41 @@
           <t>1.6</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1.166</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="n">
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J7" s="2" t="n">
+      <c r="K7" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 11</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Line integrals and surface integrals</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>5.8, 5.10</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr"/>
-      <c r="O7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -874,35 +950,45 @@
           <t>10.2</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>10.1, 10.3</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="n">
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="2" t="n">
+      <c r="K8" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Fri Nov 13</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>5.5, 5.7; App. D</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.7.1 Parts 1-4</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>WHW10</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -922,39 +1008,45 @@
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>WHW03</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Quiz 1 (Ch 1)</t>
         </is>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="J9" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J9" s="2" t="n">
+      <c r="K9" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 16</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Vector and scalar fields; the gradient</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>8.1-8.4</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
-      <c r="O9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.2.1 Parts 5-6</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -978,31 +1070,41 @@
           <t>10.2</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="n">
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="J10" s="2" t="n">
+      <c r="K10" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Wed Nov 18</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>Work, path integrals, and the gradient theorem</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>8.5</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.4.1</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1026,31 +1128,37 @@
           <t>10.10</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10.5, 10.8</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="I11" s="3" t="n">
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="J11" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="K11" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr"/>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr"/>
+      <c r="O11" s="3" t="inlineStr"/>
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>WHW11</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
@@ -1080,33 +1188,43 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
+          <t>10.216</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
           <t>WHW04</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="n">
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="J12" s="2" t="n">
+      <c r="K12" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 23</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>Divergence and curl, geometrically</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Feynman Vol II Ch 2-3</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
-      <c r="O12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1130,23 +1248,29 @@
           <t>3.1-3.4</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.2.1</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="I13" s="4" t="n"/>
+      <c r="H13" s="2" t="inlineStr"/>
       <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Wed Nov 25</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="M13" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr"/>
       <c r="N13" s="4" t="inlineStr"/>
       <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1170,23 +1294,29 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.4.1</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="I14" s="4" t="n"/>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>Fri Nov 27</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr"/>
       <c r="N14" s="4" t="inlineStr"/>
       <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1206,35 +1336,41 @@
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>WHW05</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="n">
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K15" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 30</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Divergence, curl, and the Laplacian</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>8.6-8.7</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr"/>
-      <c r="O15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.6.1 Parts 1-9</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -1252,29 +1388,35 @@
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="4" t="inlineStr"/>
-      <c r="I16" s="2" t="n">
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Wed Dec 2</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>8.9-8.10; Feynman Vol II Ch 3</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr"/>
-      <c r="O16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1298,35 +1440,45 @@
           <t>2.1-2.2</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="n">
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>Fri Dec 4</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Conservative vector fields</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>8.11</t>
         </is>
       </c>
-      <c r="N17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>WHW12</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr"/>
+      <c r="Q17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1352,33 +1504,43 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>DE 2.3.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
           <t>WHW06</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="n">
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="K18" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 7</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Introduction to Fourier series</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>9.1-9.3</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr"/>
-      <c r="O18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.2.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1402,31 +1564,41 @@
           <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2.209</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="n">
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J19" s="2" t="n">
+      <c r="K19" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Wed Dec 9</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Fourier series: different periods, finite domains, complex exponentials</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>9.4-9.5</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1450,35 +1622,45 @@
           <t>6.1-6.2</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="n">
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="K20" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Fri Dec 11</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Intro to PDEs: the heat equation; separation of variables</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>11.1-11.2, 11.4</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
         <is>
           <t>WHW13</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr"/>
+      <c r="Q20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1498,39 +1680,45 @@
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>WHW07</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="J21" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="K21" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 14</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>11.3, 9.6</t>
         </is>
       </c>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.3.1 Part 1</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1556,25 +1744,31 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
+          <t>DE 6.3.1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>Non-Newtonian Scientist due</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="I22" s="4" t="n"/>
+      <c r="H22" s="2" t="inlineStr"/>
       <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="M22" s="4" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (registrar schedules)</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
       <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr"/>
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>Final (Ch 8, 9, 11 + redemptions)</t>
         </is>
@@ -1602,8 +1796,13 @@
           <t>6.5-6.7</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.5.1</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1611,6 +1810,486 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>The following problems are useful practice for the week. I recommend starting with the warm-ups. If they're too easy, move on to Essentials. If you're interested in the Depth content, you can add those problems as well. You are not expected to do all the problems. DE x.y.1 = the Discovery Exercise of section x.y. Answers to odd problems: felderbooks.com/mathmethods (Appendix M).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>WHW</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Covers</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Warm-up</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Essentials</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Depth</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WHW01</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 11</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Intro to ODEs (1.1-1.2)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ODEs: 1.17, 1.19</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>ODEs: 1.18, 1.20, 1.21, 1.25</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>ODEs: 1.33, 1.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>WHW02</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 18</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants (1.3); separation of variables (1.5)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants: 1.39, 1.41, 1.43. Separation of variables: 1.90, 1.91, 1.93, 1.95</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants: 1.38, 1.46, 1.58. Separation of variables: 1.103</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants: 1.60. Separation of variables: 1.105</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>WHW03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 25</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check, superposition (1.6); linear operators (10.2)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check: 1.108, 1.109. Sec 10.2: 10.1, 10.3, 10.5, 10.8</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check: 1.111, 1.113, 1.117, 1.122, 1.29. Sec 10.2: 10.13, 10.26, 10.31</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check: 1.125, 1.131. Sec 10.2: 10.32, 10.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>WHW04</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 2</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ODEs in Python; Heaviside, Dirac, Laplace (10.10)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>10.216, 10.217, 10.218</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.10: 10.219, 10.223, 10.230, 10.242</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on posit.smith.edu</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>WHW05</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 9</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Solving ODEs with Laplace transforms (10.11); complex numbers and Euler (3.1-3.5)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.11: 10.246, 10.248. Complex numbers: 3.17, 3.19, 3.47. Euler / complex ODE: 3.59, 3.65, 3.92</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.11: 10.252, 10.261, 10.263, 10.264. Complex numbers: 3.49, 3.54. Euler / complex ODE: 3.77, 3.94, 3.95</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Sec 10.11: 10.270, 10.272, 10.274. Complex numbers: 3.45, 3.56. Euler / complex ODE: 3.85, 3.107</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>WHW06</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 16</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Linear approximations (2.1-2.2); Maclaurin series (2.3)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Linear approximations: 2.6, 2.7, 2.16</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin series: 2.31, 2.35, 2.37</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin series: 2.86, 2.87</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>WHW07</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 23</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series (2.4-2.5); matrices and the three-spring problem (6.1-6.2)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series: 2.41. The three-spring problem: 6.2. Normal modes: 6.3. Matrices: 6.19</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin/Taylor: 2.47, 2.49, 2.53, 2.55, 2.57, 2.67. The three-spring problem: 6.7, 6.17. Normal modes: 6.9. Matrices: 6.21, 6.23</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series: 2.71, 2.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>WHW08</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 30</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix times column, basis, matrix times matrix, identity, inverse, determinants (6.3-6.7)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix times column: 6.27, 6.29, 6.31. Matrix-matrix: 6.69. Identity and inverse: DE 6.6.1, 6.97. Determinants: 6.127, 6.129</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Matrix times column: 6.35, 6.41. Matrix-matrix: 6.81, 6.89, 6.91. Identity and inverse: 6.99, 6.101, 6.103, 6.107, 6.109, 6.119, 6.121, 6.123. Determinants: 6.133, 6.139</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Basis and transformations: 6.45, 6.53, 6.55, 6.57, 6.61. Determinants: 6.147, 6.161</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>WHW09</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 6</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvalues and eigenvectors (6.8); coupled oscillators (6.9)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvectors &amp; eigenvalues: 6.166, 6.170, 6.172, 6.175</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvectors &amp; eigenvalues: 6.171, 6.173, 6.177</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvectors &amp; eigenvalues: 6.179, 6.181, 6.185</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>WHW10</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 13</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Setting up integrals; Cartesian doubles, polar; line and surface integrals (5.1-5.4, 5.6, 5.8, 5.10)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Setting up 1D integrals: 5.1-5.3. Single integrals in multiple dimensions: 5.25, 5.27, 5.29, 5.31. Cartesian rectangular double integrals: 5.61, 5.63. Line integrals: 5.197. Surface integrals: 5.255</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Setting up 1D integrals: 5.7, 5.9, 5.11, 5.19, 5.23. Single integrals in multiple dimensions: 5.35, 5.43, 5.45, 5.51. Cartesian rectangular: 5.71, 5.75, 5.77. Cartesian non-rectangular: 5.83, 5.85, 5.97, 5.101. Line integrals: 5.199, 5.201, 5.215, 5.217, 5.229. Surface integrals: 5.256, 5.257, 5.263</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Line integrals: 5.223, 5.225, 5.235</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>WHW11</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Cylindrical and spherical coordinates (5.5, 5.7); fields, potential, gradient (8.1-8.5)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Spherical coordinates: 5.167, 5.174. Scalar and vector fields: DE 8.2.1, 8.1. Potential in 1D: DE 8.3.1, 8.29, 8.35. From potential to gradients: 8.53, 8.55</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Spherical coordinates: 5.181, 5.187. Polar and cylindrical: 5.129, 5.137, 5.147, 5.153. Scalar and vector fields: 8.5, 8.7, 8.9, 8.17, 8.19, 8.21, 8.25. Potential in 1D: 8.37, 8.41, 8.43. From potential to gradients: 8.57, 8.59, 8.65</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Polar and cylindrical: 5.157, 5.169, 5.171, 5.193. All coordinates: 5.165</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>WHW12</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 4</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl, Feynman and Felder (Feynman II 2-3, 8.6-8.7); divergence theorem and Stokes' theorem (8.9-8.10)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl by inspection: 8.84, 8.86. Divergence theorem: DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl: 8.88, 8.90, 8.94, 8.98, 8.102, 8.110. Divergence theorem: 8.147, 8.151, 8.155, 8.157. Stokes' theorem: 8.159, 8.163, 8.165, 8.169, 8.171</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>8.106. Write out Feynman's flux-through-a-tiny-cube derivation of the divergence theorem in your own words, with pictures</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>WHW13</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 11</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields (8.11); Fourier series (9.1-9.5)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields: DE 8.11.1. Fourier series: DE 9.2.1, 9.5, 9.7, 9.9</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields: 8.178. Fourier series: 9.15, 9.17, 9.23, 9.27, 9.29, 9.33</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Conservative fields: 8.173, 8.177, 8.179, 8.181. Different periods and finite domains: 9.38, 9.41, 9.47. Complex Fourier series: 9.60, 9.62, 9.66</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1627,27 +2306,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Drop</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Points Each</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Total Points</t>
         </is>

</xml_diff>

<commit_message>
F2026 calendar: dedupe WHW lists against PCCI assignments
Problems promoted to graded PCCIs are no longer repeated in the WHW
practice tiers (10.1/10.3/10.5/10.8, 10.216, 6.2, 6.166, 6.175, 5.1,
DE 8.2.1, DE 8.9.1, DE 8.11.1, DE 9.2.1); convention noted in the
generator comments. Regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1947,7 +1947,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Guess and check: 1.108, 1.109. Sec 10.2: 10.1, 10.3, 10.5, 10.8</t>
+          <t>Guess and check: 1.108, 1.109</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>10.216, 10.217, 10.218</t>
+          <t>10.217, 10.218</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Taylor series: 2.41. The three-spring problem: 6.2. Normal modes: 6.3. Matrices: 6.19</t>
+          <t>Taylor series: 2.41. Normal modes: 6.3. Matrices: 6.19</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Eigenvectors &amp; eigenvalues: 6.166, 6.170, 6.172, 6.175</t>
+          <t>Eigenvectors &amp; eigenvalues: 6.170, 6.172</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D integrals: 5.1-5.3. Single integrals in multiple dimensions: 5.25, 5.27, 5.29, 5.31. Cartesian rectangular double integrals: 5.61, 5.63. Line integrals: 5.197. Surface integrals: 5.255</t>
+          <t>Setting up 1D integrals: 5.2, 5.3. Single integrals in multiple dimensions: 5.25, 5.27, 5.29, 5.31. Cartesian rectangular double integrals: 5.61, 5.63. Line integrals: 5.197. Surface integrals: 5.255</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Spherical coordinates: 5.167, 5.174. Scalar and vector fields: DE 8.2.1, 8.1. Potential in 1D: DE 8.3.1, 8.29, 8.35. From potential to gradients: 8.53, 8.55</t>
+          <t>Spherical coordinates: 5.167, 5.174. Scalar and vector fields: 8.1. Potential in 1D: DE 8.3.1, 8.29, 8.35. From potential to gradients: 8.53, 8.55</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Divergence and curl by inspection: 8.84, 8.86. Divergence theorem: DE 8.9.1</t>
+          <t>Divergence and curl by inspection: 8.84, 8.86</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Conservative fields: DE 8.11.1. Fourier series: DE 9.2.1, 9.5, 9.7, 9.9</t>
+          <t>Fourier series: 9.5, 9.7, 9.9</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
F2026 calendar: no PCCI on day 1; first PCCI (syllabus+advice) day 2
Nobody has the syllabus before the first class. Matches Gary's actual
pattern (first PCCI on day 2). DE 1.2.1 dropped rather than shifted:
class 01 does its content live. DE 1.3.1 unchanged on Mon Sep 14,
still priming the arbitrary-constants day. 34 PCCIs.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -586,11 +586,7 @@
           <t>1.1-1.2</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
@@ -650,7 +646,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>DE 1.2.1</t>
+          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Grading rebalance: participation 2 pts/day (70), quizzes 140, final 185
Michael's 2026-08-25 decision, made in the syllabus: more credit for
attendance/participation. Generator constants updated (asserts still
require exactly 1000), xlsx regenerated, MoodleBuildSpec gradebook
and TODO item 8 synced.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -2341,7 +2341,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <f>(B2-C2)*D2</f>
@@ -2402,7 +2402,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E5">
         <f>(B5-C5)*D5</f>
@@ -2422,7 +2422,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="E6">
         <f>(B6-C6)*D6</f>

</xml_diff>

<commit_message>
Calendar: single-block 'Schedule (web)' tab for the Moodle embed
The two-block Schedule sheet is ~1600px wide; the embed needs one
continuous ~800px table.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule (web)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1811,6 +1812,1350 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Topics</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Reading Due</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>HW Due</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Exams</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 9</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Syllabus; SHO and overview of differential equations</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1.1-1.2</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 11</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Generating ODEs from physical situations</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1.1-1.2</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>WHW01</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Mon Sep 14</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Arbitrary constants; initial conditions</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.3.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 16</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Separation of variables</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.5.1 Parts 1-5</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Fri Sep 18</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Guess and check</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>DE 1.6.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>WHW02</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Mon Sep 21</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Linearity, homogeneity, superposition</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1.166</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 23</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Methods of solving ODEs: guess and check</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>10.1, 10.3</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Fri Sep 25</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 1 (Ch 1)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>WHW03</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 1 (Ch 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Jupyter notebook exercise: ODEs in Python</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>10.2</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Wed Sep 30</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Heaviside, Dirac delta, and the Laplace transform</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>10.10</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>10.5, 10.8</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 2</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Using Laplace transforms to solve ODEs</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>10.11</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>10.216</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>WHW04</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Mon Oct 5</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Complex numbers: basic properties</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>3.1-3.4</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.2.1</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Euler's formula; complex ODEs</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>DE 3.4.1</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 9</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Flex day (snow / Mountain Day buffer)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>WHW05</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Mon Oct 12</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>No class - Autumn recess</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 14</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Linear approximations</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2.1-2.2</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 16</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Maclaurin series</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.3.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>WHW06</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Mon Oct 19</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Taylor series; finding one series from another</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2.4-2.5 (convergence: App. C)</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2.209</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 21</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Properties of matrices</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>6.1-6.2</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Fri Oct 23</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 2 (Ch 10, 3, 2)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>WHW07</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 2 (Ch 10, 3, 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Mon Oct 26</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Matrix x column; vector transformations</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>6.3-6.4</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.3.1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 28</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Matrix multiplication; identity, determinant, inverse</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>6.5-6.7</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.5.1</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Fri Oct 30</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Finding eigenvalues and eigenvectors</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>DE 6.8.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>WHW08</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 2</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Eigenvalues and eigenvectors, continued</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>6.8</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>6.166</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 4</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>The two-coupled-oscillator problem</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>6.175</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 6</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Setting up 1D and 2D integrals</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>5.1-5.2</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>WHW09</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 9</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Cartesian 2D integrals; polar coordinates</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>5.3-5.4, 5.6</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.4.1</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 11</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Line integrals and surface integrals</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>5.8, 5.10</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Fri Nov 13</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>5.5, 5.7; App. D</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.7.1 Parts 1-4</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>WHW10</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 16</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Vector and scalar fields; the gradient</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>8.1-8.4</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.2.1 Parts 5-6</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 18</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Work, path integrals, and the gradient theorem</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.4.1</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Fri Nov 20</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 3 (Ch 6, 5)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>WHW11</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Quiz 3 (Ch 6, 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 23</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Divergence and curl, geometrically</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Feynman Vol II Ch 2-3</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Wed Nov 25</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>No class - Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr"/>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Fri Nov 27</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>No class - Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
+      <c r="H36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Mon Nov 30</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Divergence, curl, and the Laplacian</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>8.6-8.7</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.6.1 Parts 1-9</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Wed Dec 2</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Divergence theorem; Stokes' theorem</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>8.9-8.10; Feynman Vol II Ch 3</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 4</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Conservative vector fields</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>8.11</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>WHW12</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Mon Dec 7</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Introduction to Fourier series</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>9.1-9.3</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.2.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Wed Dec 9</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Fourier series: different periods, finite domains, complex exponentials</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>9.4-9.5</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 11</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>11.1-11.2, 11.4</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>WHW13</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Mon Dec 14</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Normal modes of the wave equation; Fourier transforms</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>11.3, 9.6</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.3.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Sat Dec 19</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Final exam period Dec 19-22 (registrar schedules)</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Final (Ch 8, 9, 11 + redemptions)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2285,7 +3630,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Calendar: chunked Schedule (web) tab for the half-semester embed
Two chunks split at fall break, each with its own header row; the
generator prints the embed ranges every run. Spec gains the full
embed/switch/re-import procedure.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1812,7 +1812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2310,97 +2310,109 @@
       <c r="H16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 14</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Linear approximations</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>2.1-2.2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>DE 2.2.1 Parts 1-5</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Topics</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Reading Due</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>PCCI</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>HW Due</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>Exams</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Fri Oct 16</t>
+          <t>Wed Oct 14</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Maclaurin series</t>
+          <t>Linear approximations</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.1-2.2</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>DE 2.3.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>WHW06</t>
-        </is>
-      </c>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Mon Oct 19</t>
+          <t>Fri Oct 16</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Taylor series; finding one series from another</t>
+          <t>Maclaurin series</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5 (convergence: App. C)</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2.209</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
+          <t>DE 2.3.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>WHW06</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -2408,123 +2420,123 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 21</t>
+          <t>Mon Oct 19</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Properties of matrices</t>
+          <t>Taylor series; finding one series from another</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>6.1-6.2</t>
+          <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>2.209</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
       <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Wed Oct 21</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Properties of matrices</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>6.1-6.2</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Fri Oct 23</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>WHW07</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 26</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Matrix x column; vector transformations</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>6.3-6.4</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.3.1</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Non-Newtonian Scientist due</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Wed Oct 28</t>
+          <t>Mon Oct 26</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Matrix multiplication; identity, determinant, inverse</t>
+          <t>Matrix x column; vector transformations</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.5-6.7</t>
+          <t>6.3-6.4</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>DE 6.5.1</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
+          <t>DE 6.3.1</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2532,50 +2544,46 @@
         <v>8</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Fri Oct 30</t>
+          <t>Wed Oct 28</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Finding eigenvalues and eigenvectors</t>
+          <t>Matrix multiplication; identity, determinant, inverse</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>6.5-6.7</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>DE 6.8.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>WHW08</t>
-        </is>
-      </c>
+          <t>DE 6.5.1</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
       <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Mon Nov 2</t>
+          <t>Fri Oct 30</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Eigenvalues and eigenvectors, continued</t>
+          <t>Finding eigenvalues and eigenvectors</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2585,10 +2593,14 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>6.166</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
+          <t>DE 6.8.1 Parts 1-3</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>WHW08</t>
+        </is>
+      </c>
       <c r="H25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
@@ -2596,26 +2608,26 @@
         <v>9</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 4</t>
+          <t>Mon Nov 2</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>The two-coupled-oscillator problem</t>
+          <t>Eigenvalues and eigenvectors, continued</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>6.9</t>
+          <t>6.8</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>6.175</t>
+          <t>6.166</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -2626,63 +2638,63 @@
         <v>9</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Fri Nov 6</t>
+          <t>Wed Nov 4</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>The two-coupled-oscillator problem</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
+          <t>6.9</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>WHW09</t>
-        </is>
-      </c>
+          <t>6.175</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Mon Nov 9</t>
+          <t>Fri Nov 6</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals; polar coordinates</t>
+          <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4, 5.6</t>
+          <t>5.1-5.2</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>DE 5.4.1</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>WHW09</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2690,26 +2702,26 @@
         <v>10</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 11</t>
+          <t>Mon Nov 9</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>Cartesian 2D integrals; polar coordinates</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
+          <t>5.3-5.4, 5.6</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>5.163 parts a and d</t>
+          <t>DE 5.4.1</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -2720,63 +2732,63 @@
         <v>10</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Fri Nov 13</t>
+          <t>Wed Nov 11</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>5.5, 5.7; App. D</t>
+          <t>5.8, 5.10</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DE 5.7.1 Parts 1-4</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>WHW10</t>
-        </is>
-      </c>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
       <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Mon Nov 16</t>
+          <t>Fri Nov 13</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; the gradient</t>
+          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.4</t>
+          <t>5.5, 5.7; App. D</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DE 8.2.1 Parts 5-6</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
+          <t>DE 5.7.1 Parts 1-4</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>WHW10</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
@@ -2784,115 +2796,127 @@
         <v>11</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Wed Nov 18</t>
+          <t>Mon Nov 16</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Work, path integrals, and the gradient theorem</t>
+          <t>Vector and scalar fields; the gradient</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.1-8.4</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>DE 8.4.1</t>
+          <t>DE 8.2.1 Parts 5-6</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
       <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Wed Nov 18</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Work, path integrals, and the gradient theorem</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>8.5</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>DE 8.4.1</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>WHW11</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
+    <row r="35">
+      <c r="A35" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Mon Nov 23</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Divergence and curl, geometrically</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Feynman Vol II Ch 2-3</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Wed Nov 25</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>No class - Thanksgiving</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
       <c r="B36" s="4" t="n"/>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Fri Nov 27</t>
+          <t>Wed Nov 25</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2906,60 +2930,48 @@
       <c r="H36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 30</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Divergence, curl, and the Laplacian</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>8.6-8.7</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.6.1 Parts 1-9</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Fri Nov 27</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>No class - Thanksgiving</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Wed Dec 2</t>
+          <t>Mon Nov 30</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Divergence theorem; Stokes' theorem</t>
+          <t>Divergence, curl, and the Laplacian</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10; Feynman Vol II Ch 3</t>
+          <t>8.6-8.7</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DE 8.9.1</t>
+          <t>DE 8.6.1 Parts 1-9</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -2970,63 +2982,63 @@
         <v>13</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Fri Dec 4</t>
+          <t>Wed Dec 2</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Conservative vector fields</t>
+          <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>8.9-8.10; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>WHW12</t>
-        </is>
-      </c>
+          <t>DE 8.9.1</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Mon Dec 7</t>
+          <t>Fri Dec 4</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Introduction to Fourier series</t>
+          <t>Conservative vector fields</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.3</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>DE 9.2.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr"/>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>WHW12</t>
+        </is>
+      </c>
       <c r="H40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
@@ -3034,26 +3046,26 @@
         <v>14</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Wed Dec 9</t>
+          <t>Mon Dec 7</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains, complex exponentials</t>
+          <t>Introduction to Fourier series</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>9.4-9.5</t>
+          <t>9.1-9.3</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>DE 9.4.1 Part 1</t>
+          <t>DE 9.2.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
@@ -3064,82 +3076,112 @@
         <v>14</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Fri Dec 11</t>
+          <t>Wed Dec 9</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation; separation of variables</t>
+          <t>Fourier series: different periods, finite domains, complex exponentials</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2, 11.4</t>
+          <t>9.4-9.5</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>DE 11.2.1 Parts 1-2</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>WHW13</t>
-        </is>
-      </c>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Fri Dec 11</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>11.1-11.2, 11.4</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>WHW13</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B43" s="2" t="n">
+      <c r="B44" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Mon Dec 14</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>11.3, 9.6</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>DE 11.3.1 Part 1</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (registrar schedules)</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr"/>
-      <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr">
         <is>
           <t>Final (Ch 8, 9, 11 + redemptions)</t>
         </is>

</xml_diff>

<commit_message>
Calendar: one canonical Schedule tab (chunked single block)
Drop the two-side-by-side-blocks print layout -- it existed to serve
the embed-half-at-a-time practice, which the chunked ranges now do.
Header cells wrap; Week/Class/Reading Due columns widened.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -8,9 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule (web)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WHW Problem Lists" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grade Categories" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -81,9 +80,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -96,6 +97,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -462,1364 +464,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="6" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Topics</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Reading Due</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>PCCI</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>HW Due</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Exams</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Topics</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Reading Due</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>PCCI</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>HW Due</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Exams</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 9</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Syllabus; SHO and overview of differential equations</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1.1-1.2</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 30</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Finding eigenvalues and eigenvectors</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.8.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>WHW08</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Fri Sep 11</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Generating ODEs from physical situations</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>1.1-1.2</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Read the syllabus and the advice from former students; bring one question or comment</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>WHW01</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 2</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Eigenvalues and eigenvectors, continued</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>6.8</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>6.166</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Mon Sep 14</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Arbitrary constants; initial conditions</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>DE 1.3.1 Part 1</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K4" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Wed Nov 4</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>The two-coupled-oscillator problem</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>6.9</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>6.175</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 16</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Separation of variables</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>DE 1.5.1 Parts 1-5</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Fri Nov 6</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Setting up 1D and 2D integrals</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>5.1-5.2</t>
-        </is>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
-        <is>
-          <t>WHW09</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Fri Sep 18</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Guess and check</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>DE 1.6.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>WHW02</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K6" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 9</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Cartesian 2D integrals; polar coordinates</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>5.3-5.4, 5.6</t>
-        </is>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>DE 5.4.1</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr"/>
-      <c r="Q6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Mon Sep 21</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Linearity, homogeneity, superposition</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>1.166</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Wed Nov 11</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Line integrals and surface integrals</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>5.8, 5.10</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>5.163 parts a and d</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 23</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Methods of solving ODEs: guess and check</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>10.1, 10.3</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Fri Nov 13</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>5.5, 5.7; App. D</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>DE 5.7.1 Parts 1-4</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>WHW10</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Fri Sep 25</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 1 (Ch 1)</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>WHW03</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 1 (Ch 1)</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 16</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Vector and scalar fields; the gradient</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>8.1-8.4</t>
-        </is>
-      </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.2.1 Parts 5-6</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Mon Sep 28</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Jupyter notebook exercise: ODEs in Python</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="K10" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Wed Nov 18</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Work, path integrals, and the gradient theorem</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>8.5</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.4.1</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr"/>
-      <c r="Q10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 30</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Heaviside, Dirac delta, and the Laplace transform</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>10.10</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>10.5, 10.8</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="J11" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>Fri Nov 20</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 3 (Ch 6, 5)</t>
-        </is>
-      </c>
-      <c r="N11" s="3" t="inlineStr"/>
-      <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="3" t="inlineStr">
-        <is>
-          <t>WHW11</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 3 (Ch 6, 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 2</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Using Laplace transforms to solve ODEs</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>10.11</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>10.216</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>WHW04</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="K12" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 23</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Divergence and curl, geometrically</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>Feynman Vol II Ch 2-3</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>Read Feynman II Ch 2; write one sentence on what the gradient of temperature means physically</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr"/>
-      <c r="Q12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 5</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Complex numbers: basic properties</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>3.1-3.4</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>DE 3.2.1</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>Wed Nov 25</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>No class - Thanksgiving</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr"/>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 7</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Euler's formula; complex ODEs</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>3.5</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>DE 3.4.1</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Fri Nov 27</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>No class - Thanksgiving</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
-      <c r="Q14" s="4" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 9</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Flex day (snow / Mountain Day buffer)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>WHW05</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="J15" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K15" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Mon Nov 30</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Divergence, curl, and the Laplacian</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>8.6-8.7</t>
-        </is>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.6.1 Parts 1-9</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Mon Oct 12</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>No class - Autumn recess</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="J16" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K16" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Wed Dec 2</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Divergence theorem; Stokes' theorem</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>8.9-8.10; Feynman Vol II Ch 3</t>
-        </is>
-      </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.9.1</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr"/>
-      <c r="Q16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 14</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Linear approximations</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>2.1-2.2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>DE 2.2.1 Parts 1-5</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="K17" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Fri Dec 4</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Conservative vector fields</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>8.11</t>
-        </is>
-      </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
-        <is>
-          <t>WHW12</t>
-        </is>
-      </c>
-      <c r="Q17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Fri Oct 16</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Maclaurin series</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>DE 2.3.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>WHW06</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Mon Dec 7</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>Introduction to Fourier series</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>9.1-9.3</t>
-        </is>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>DE 9.2.1 Parts 1-3</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr"/>
-      <c r="Q18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 19</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Taylor series; finding one series from another</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>2.4-2.5 (convergence: App. C)</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>2.209</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K19" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Wed Dec 9</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>Fourier series: different periods, finite domains, complex exponentials</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>9.4-9.5</t>
-        </is>
-      </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>DE 9.4.1 Part 1</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 21</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Properties of matrices</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>6.1-6.2</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>6.2</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="K20" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Fri Dec 11</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Intro to PDEs: the heat equation; separation of variables</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>11.1-11.2, 11.4</t>
-        </is>
-      </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>DE 11.2.1 Parts 1-2</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>WHW13</t>
-        </is>
-      </c>
-      <c r="Q20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Fri Oct 23</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 2 (Ch 10, 3, 2)</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>WHW07</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Quiz 2 (Ch 10, 3, 2)</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K21" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>Mon Dec 14</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Normal modes of the wave equation; Fourier transforms</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr">
-        <is>
-          <t>11.3, 9.6</t>
-        </is>
-      </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>DE 11.3.1 Part 1</t>
-        </is>
-      </c>
-      <c r="P21" s="2" t="inlineStr"/>
-      <c r="Q21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Mon Oct 26</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Matrix x column; vector transformations</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>6.3-6.4</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.3.1</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Non-Newtonian Scientist due</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="J22" s="4" t="n"/>
-      <c r="K22" s="4" t="n"/>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>Sat Dec 19</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>Final exam period Dec 19-22 (registrar schedules)</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
-      <c r="Q22" s="4" t="inlineStr">
-        <is>
-          <t>Final (Ch 8, 9, 11 + redemptions)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Wed Oct 28</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Matrix multiplication; identity, determinant, inverse</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>6.5-6.7</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.5.1</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -3192,7 +1844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3217,32 +1869,32 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>WHW</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Covers</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Warm-up</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Depth</t>
         </is>
@@ -3672,7 +2324,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3689,27 +2341,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Drop</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Points Each</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Total Points</t>
         </is>

</xml_diff>

<commit_message>
Platform: jupyterhub.smith.edu replaces posit (syllabus, generator, spec, notes)
Same switch as PHY 317 (2026-09-07): posit's Workbench cannot start
sessions and has no packages; the hub has the full stack and ipywidgets.
Syllabus (two places), the Sep 28 PCCI and WHW04 depth item in the
generator, MoodleBuildSpec (with the hub lessons: VPN off campus, pin
%matplotlib inline because the hub defaults to ipympl), TODO item 27
resolved, ComputationalProblems.md's scipy caveat lifted (scipy 1.14 is
there), Notebooks2026 README.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Log into posit.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
+          <t>Log into jupyterhub.smith.edu and open a blank Jupyter notebook; bring your laptop</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Redo the class notebook's exercises from scratch in a fresh notebook on posit.smith.edu</t>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WHW01: 1.36 (by computer) moved to WHW04; guard against by-computer problems before the Python class
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1928,7 +1928,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>ODEs: 1.33, 1.36</t>
+          <t>ODEs: 1.33</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu</t>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu. Sec 1.2: 1.36 (compound interest, by computer; moved here from WHW01)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WHW01 records the set that was actually delivered (1.36 kept, with its skip clause)
The 2026-09-11 fix took 1.36 off WHW01, but the Moodle page was never
edited, so the set students submitted on Mon Sep 14 still carried it. A
delivered set is a record, not a plan, so the calendar now shows what
they got and the by-computer guard exempts delivered sets. 1.36 stays on
WHW04 as well, reworded from 'moved here' to a second offering now that
they have Python.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RAcPZi5nkqZkcCQ9LAREd
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1928,7 +1928,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>ODEs: 1.33</t>
+          <t>ODEs: 1.33, 1.36 (if you don't have experience with computational tools, feel free to completely skip this)</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu. Sec 1.2: 1.36 (compound interest, by computer; moved here from WHW01)</t>
+          <t>Redo the class notebook's exercises from scratch in a fresh notebook on jupyterhub.smith.edu. Sec 1.2: 1.36 (compound interest, by computer; it was optional Depth on WHW01 before we had Python, so here it is with the tools)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 2026-09-19: reading splits for two dead PCCIs, chapter-card comma bug, two-star guard, stale grading text
- make_fall2026_calendar.py: Oct 5/7 readings 3.1-3.3 / 3.4-3.5 and Nov
  16/18 readings 8.1-8.3 / 8.4-8.5 so DE 3.4.1 and DE 8.4.1 are not read
  before their PCCI day (playbook 6a).
- make_chapter_slides.py: split tier text on commas outside parentheses.
- make_active_learning.py: two-star budget warning (parity with 317).
- README.md: current grading scheme (was the Aug 11 draft).
- TODO.md: item 35 closed; item 33 names the calendar label, not a Page.
- MoodleBuildSpec.md: calendar embed is a label.
- Regenerated xlsx.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -876,7 +876,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>3.1-3.4</t>
+          <t>3.1-3.3</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>3.4-3.5</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1457,12 +1457,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; the gradient</t>
+          <t>Vector and scalar fields; potential</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.4</t>
+          <t>8.1-8.3</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1487,12 +1487,12 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Work, path integrals, and the gradient theorem</t>
+          <t>The gradient; work, path integrals, and the gradient theorem</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.4-8.5</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
210 calendar rebuilt on Manbir's actual S26 meetings; Mountain Day recorded
Mountain Day (Wed Sep 23) was never entered here (317's calendar was), so
class 07 (Felder 10.2) silently vanished. It is now a cancelled slot (class
numbers unchanged) and 10.2 is dropped. The flex day is gone (Mountain Day
spent it). From Oct 2 on each meeting is Manbir's actual S26 meeting, quiz
dates fixed; PCCIs moved with their topics; Feynman is woven into the six
vector-calculus days; Dec 14 is the fixed finale.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -717,14 +717,10 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Methods of solving ODEs: guess and check</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>10.2</t>
-        </is>
-      </c>
+          <t>Mountain Day (no class)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>10.1, 10.3</t>
@@ -931,11 +927,19 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Flex day (snow / Mountain Day buffer)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
+          <t>Linear approximations</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2.1-2.2</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>DE 2.2.1 Parts 1-5</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>WHW05</t>
@@ -1017,17 +1021,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Linear approximations</t>
+          <t>Maclaurin series</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2.1-2.2</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>DE 2.2.1 Parts 1-5</t>
+          <t>DE 2.3.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
@@ -1047,17 +1051,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Maclaurin series</t>
+          <t>Taylor series; finding one series from another</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.4-2.5 (convergence: App. C)</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>DE 2.3.1 Parts 1-3</t>
+          <t>2.209</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1081,17 +1085,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Taylor series; finding one series from another</t>
+          <t>Properties of matrices</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5 (convergence: App. C)</t>
+          <t>6.1-6.2</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2.209</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
@@ -1111,17 +1115,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Properties of matrices</t>
+          <t>Matrix x column; vector transformations</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>6.1-6.2</t>
+          <t>6.3-6.4</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>DE 6.3.1</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
@@ -1171,17 +1175,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Matrix x column; vector transformations</t>
+          <t>Matrix multiplication; identity and inverse</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.3-6.4</t>
+          <t>6.5-6.6</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>DE 6.3.1</t>
+          <t>DE 6.5.1</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1205,17 +1209,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Matrix multiplication; identity, determinant, inverse</t>
+          <t>Determinants; finding eigenvalues and eigenvectors</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>6.5-6.7</t>
+          <t>6.7-6.8</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>DE 6.5.1</t>
+          <t>DE 6.8.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1235,17 +1239,17 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Finding eigenvalues and eigenvectors</t>
+          <t>Eigenvectors; the two-coupled-oscillator problem</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>6.8-6.9</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>DE 6.8.1 Parts 1-3</t>
+          <t>6.166</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1269,17 +1273,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Eigenvalues and eigenvectors, continued</t>
+          <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>6.8</t>
+          <t>5.1-5.2</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>6.166</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1299,17 +1303,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>The two-coupled-oscillator problem</t>
+          <t>Cartesian 2D integrals</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>6.9</t>
+          <t>5.3-5.4</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>6.175</t>
+          <t>DE 5.4.1</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1329,19 +1333,15 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>Polar coordinates</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
@@ -1363,17 +1363,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals; polar coordinates</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4, 5.6</t>
+          <t>5.8, 5.10</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>DE 5.4.1</t>
+          <t>5.163 parts a and d</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1393,17 +1393,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>Cylindrical and spherical coordinates</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
+          <t>5.5, 5.7; App. D</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>5.163 parts a and d</t>
+          <t>DE 5.7.1 Parts 1-4</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1423,17 +1423,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Coordinate systems: cylindrical and spherical (review + practice)</t>
+          <t>Vector and scalar fields; potential</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>5.5, 5.7; App. D</t>
+          <t>8.1-8.3</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DE 5.7.1 Parts 1-4</t>
+          <t>DE 8.2.1 Parts 5-6</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1457,17 +1457,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; potential</t>
+          <t>The gradient; equipotentials</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.3</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>DE 8.2.1 Parts 5-6</t>
+          <t>DE 8.4.1</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -1487,17 +1487,17 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>The gradient; work, path integrals, and the gradient theorem</t>
+          <t>Potential from a field; the gradient theorem; divergence and curl (Feynman)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>8.4-8.5</t>
+          <t>8.5-8.6; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>DE 8.4.1</t>
+          <t>Read Feynman II Ch 3 sections 3-1 to 3-6; in one or two sentences, what does the flux of a vector field out of a tiny box measure, and what does the circulation around a tiny loop measure?</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -1547,17 +1547,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Divergence and curl, geometrically</t>
+          <t>Divergence, curl, and the Laplacian; the divergence theorem</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Feynman Vol II Ch 2-3</t>
+          <t>8.6-8.7, 8.9; Feynman Vol II Ch 2</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Read Feynman II Ch 3 sections 3-1 to 3-6; in one or two sentences, what does the flux of a vector field out of a tiny box measure, and what does the circulation around a tiny loop measure?</t>
+          <t>DE 8.6.1 Parts 1-9</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -1613,17 +1613,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Divergence, curl, and the Laplacian</t>
+          <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8.6-8.7</t>
+          <t>8.9-8.10</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DE 8.6.1 Parts 1-9</t>
+          <t>DE 8.9.1</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -1643,17 +1643,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Divergence theorem; Stokes' theorem</t>
+          <t>Conservative vector fields</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10; Feynman Vol II Ch 3</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>DE 8.9.1</t>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
@@ -1673,17 +1673,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Conservative vector fields</t>
+          <t>Introduction to Fourier series</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>9.1-9.3</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+          <t>DE 9.2.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1707,17 +1707,17 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Introduction to Fourier series</t>
+          <t>Fourier series: different periods, finite domains</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.3</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>DE 9.2.1 Parts 1-3</t>
+          <t>DE 9.4.1 Part 1</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
@@ -1737,19 +1737,15 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains, complex exponentials</t>
+          <t>Fourier series with complex exponentials</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>9.4-9.5</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>DE 9.4.1 Part 1</t>
-        </is>
-      </c>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
210 calendar: class numbers count meetings held, as in 317
Mountain Day (Wed Sep 23) becomes a NO_CLASS row ("Mountain Day!!", 317's
wording) instead of a cancelled slot that kept class number 07, so Sep 25
is class 07 and the term has 38 numbered meetings. Quizzes are now keyed
by date (QUIZZES, mirroring 317's EXAMS) so a lost meeting cannot shift
them; make_review_checklists and make_chapter_slides read the new table.
The collected Sep 23 PCCI (10.1, 10.3) moves to PCCI_LOST, which the
Moodle builders read so its solution Page keeps a heading.

FLAG: the participation category still says 39 meetings x 2 pts with 4
drops; 38 were held. Michael's call.

renumber_packs_2026-10-04.py is the one-shot that renames the prep packs
08..39 -> 07..38 (dry run by default; --apply to act).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -45,12 +45,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -704,56 +704,48 @@
       <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n"/>
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Wed Sep 23</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Mountain Day!!</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B9" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Wed Sep 23</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Mountain Day (no class)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>10.1, 10.3</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Fri Sep 25</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Quiz 1 (Ch 1)</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>WHW03</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Quiz 1 (Ch 1)</t>
         </is>
@@ -764,7 +756,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -794,7 +786,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -824,7 +816,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -858,7 +850,7 @@
         <v>5</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -888,7 +880,7 @@
         <v>5</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -918,7 +910,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -948,22 +940,22 @@
       <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="A16" s="3" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Mon Oct 12</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>No class - Autumn recess</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -1012,7 +1004,7 @@
         <v>6</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
@@ -1042,7 +1034,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
@@ -1076,7 +1068,7 @@
         <v>7</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -1106,7 +1098,7 @@
         <v>7</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -1132,30 +1124,30 @@
       <c r="H21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B22" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="B22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Fri Oct 23</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>WHW07</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Quiz 2 (Ch 10, 3, 2)</t>
         </is>
@@ -1166,7 +1158,7 @@
         <v>8</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -1200,7 +1192,7 @@
         <v>8</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -1230,7 +1222,7 @@
         <v>8</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -1264,7 +1256,7 @@
         <v>9</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -1294,7 +1286,7 @@
         <v>9</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
@@ -1324,7 +1316,7 @@
         <v>9</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
@@ -1354,7 +1346,7 @@
         <v>10</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
@@ -1384,7 +1376,7 @@
         <v>10</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
@@ -1414,7 +1406,7 @@
         <v>10</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
@@ -1448,7 +1440,7 @@
         <v>11</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -1478,7 +1470,7 @@
         <v>11</v>
       </c>
       <c r="B33" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
@@ -1504,30 +1496,30 @@
       <c r="H33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B34" s="3" t="n">
-        <v>31</v>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="B34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Fri Nov 20</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>WHW11</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>Quiz 3 (Ch 6, 5)</t>
         </is>
@@ -1538,7 +1530,7 @@
         <v>12</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
@@ -1564,47 +1556,47 @@
       <c r="H35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="A36" s="3" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Wed Nov 25</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr"/>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Fri Nov 27</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>No class - Thanksgiving</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr"/>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr"/>
+      <c r="H37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
@@ -1634,7 +1626,7 @@
         <v>13</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
@@ -1664,7 +1656,7 @@
         <v>13</v>
       </c>
       <c r="B40" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
@@ -1698,7 +1690,7 @@
         <v>14</v>
       </c>
       <c r="B41" s="2" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
@@ -1728,7 +1720,7 @@
         <v>14</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -1754,7 +1746,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
@@ -1788,7 +1780,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
@@ -1814,22 +1806,22 @@
       <c r="H44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="A45" s="3" t="n"/>
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Sat Dec 19</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>Final exam period Dec 19-22 (registrar schedules)</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr"/>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr"/>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>Final (Ch 8, 9, 11 + redemptions)</t>
         </is>

</xml_diff>

<commit_message>
210 calendar: class 13 ran ahead (the Maclaurin machine done Oct 9); class 14 = Maclaurin in Python + Taylor + series from a series (2.3-2.5), laptop day Oct 14, PCCI 2.30 (Michael, 2026-10-09)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Linear approximations</t>
+          <t>Linear approximations; the Maclaurin machine</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1013,17 +1013,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Maclaurin series</t>
+          <t>Maclaurin series in Python; Taylor series; series from a series [BRING LAPTOP]</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.3-2.5</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>DE 2.3.1 Parts 1-3</t>
+          <t>2.30 (a)-(e)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
210 calendar: slip after class 14 (a day ahead; Taylor done Oct 14): classes 16-38 one meeting earlier, flex day Mon Dec 14; xlsx regenerated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1043,17 +1043,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Taylor series; finding one series from another</t>
+          <t>Properties of matrices</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.4-2.5 (convergence: App. C)</t>
+          <t>6.1-6.2</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2.209</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1077,17 +1077,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Properties of matrices</t>
+          <t>Matrix x column; vector transformations</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>6.1-6.2</t>
+          <t>6.3-6.4</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>DE 6.3.1</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
@@ -1107,17 +1107,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Matrix x column; vector transformations</t>
+          <t>Matrix multiplication; identity and inverse</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>6.3-6.4</t>
+          <t>6.5-6.6</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>DE 6.3.1</t>
+          <t>DE 6.5.1</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
@@ -1167,17 +1167,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Matrix multiplication; identity and inverse</t>
+          <t>Determinants; finding eigenvalues and eigenvectors</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.5-6.6</t>
+          <t>6.7-6.8</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>DE 6.5.1</t>
+          <t>DE 6.8.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1201,17 +1201,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Determinants; finding eigenvalues and eigenvectors</t>
+          <t>Eigenvectors; the two-coupled-oscillator problem</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>6.7-6.8</t>
+          <t>6.8-6.9</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>DE 6.8.1 Parts 1-3</t>
+          <t>6.166</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1231,17 +1231,17 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Eigenvectors; the two-coupled-oscillator problem</t>
+          <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>6.8-6.9</t>
+          <t>5.1-5.2</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>6.166</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1265,17 +1265,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>Cartesian 2D integrals</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
+          <t>5.3-5.4</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>DE 5.4.1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1295,19 +1295,15 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals</t>
+          <t>Polar coordinates</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>DE 5.4.1</t>
-        </is>
-      </c>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
@@ -1325,15 +1321,19 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Polar coordinates</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5.6</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>5.8, 5.10</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>5.163 parts a and d</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
@@ -1355,17 +1355,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>Cylindrical and spherical coordinates</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
+          <t>5.5, 5.7; App. D</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>5.163 parts a and d</t>
+          <t>DE 5.7.1 Parts 1-4</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1385,17 +1385,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Cylindrical and spherical coordinates</t>
+          <t>Vector and scalar fields; potential</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>5.5, 5.7; App. D</t>
+          <t>8.1-8.3</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DE 5.7.1 Parts 1-4</t>
+          <t>DE 8.2.1 Parts 5-6</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1415,17 +1415,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; potential</t>
+          <t>The gradient; equipotentials</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.3</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DE 8.2.1 Parts 5-6</t>
+          <t>DE 8.4.1</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1449,17 +1449,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>The gradient; equipotentials</t>
+          <t>Potential from a field; the gradient theorem; divergence and curl (Feynman)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.5-8.6; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>DE 8.4.1</t>
+          <t>Read Feynman II Ch 3 sections 3-1 to 3-6; in one or two sentences, what does the flux of a vector field out of a tiny box measure, and what does the circulation around a tiny loop measure?</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -1479,17 +1479,17 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Potential from a field; the gradient theorem; divergence and curl (Feynman)</t>
+          <t>Divergence, curl, and the Laplacian; the divergence theorem</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>8.5-8.6; Feynman Vol II Ch 3</t>
+          <t>8.6-8.7, 8.9; Feynman Vol II Ch 2</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Read Feynman II Ch 3 sections 3-1 to 3-6; in one or two sentences, what does the flux of a vector field out of a tiny box measure, and what does the circulation around a tiny loop measure?</t>
+          <t>DE 8.6.1 Parts 1-9</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -1539,17 +1539,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Divergence, curl, and the Laplacian; the divergence theorem</t>
+          <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>8.6-8.7, 8.9; Feynman Vol II Ch 2</t>
+          <t>8.9-8.10</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>DE 8.6.1 Parts 1-9</t>
+          <t>DE 8.9.1</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -1605,17 +1605,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Divergence theorem; Stokes' theorem</t>
+          <t>Conservative vector fields</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DE 8.9.1</t>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -1635,17 +1635,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Conservative vector fields</t>
+          <t>Introduction to Fourier series</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>9.1-9.3</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+          <t>DE 9.2.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
@@ -1665,17 +1665,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Introduction to Fourier series</t>
+          <t>Fourier series: different periods, finite domains</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.3</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>DE 9.2.1 Parts 1-3</t>
+          <t>DE 9.4.1 Part 1</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1699,19 +1699,15 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains</t>
+          <t>Fourier series with complex exponentials</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>9.4</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>DE 9.4.1 Part 1</t>
-        </is>
-      </c>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr"/>
     </row>
@@ -1729,15 +1725,19 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Fourier series with complex exponentials</t>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
+          <t>11.1-11.2, 11.4</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.2.1 Parts 1-2</t>
+        </is>
+      </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
     </row>
@@ -1755,17 +1755,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation; separation of variables</t>
+          <t>Normal modes of the wave equation; Fourier transforms</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2, 11.4</t>
+          <t>11.3, 9.6</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>DE 11.2.1 Parts 1-2</t>
+          <t>DE 11.3.1 Part 1</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -1789,19 +1789,11 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Normal modes of the wave equation; Fourier transforms</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>11.3, 9.6</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>DE 11.3.1 Part 1</t>
-        </is>
-      </c>
+          <t>Flex (freed when 2026-10-14 got a day ahead: a day ahead: Michael's two-day series plan put Taylor, the SymPy notebook and the crystal on Wed Oct 14 (class 14); Friday's content was covered (decided 2026-10-12 on the assumption that Wednesday lands))</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Non-Newtonian Scientist due Wed Oct 28, not Mon Oct 26 (Michael moved it on Moodle, 2026-10-26)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>6.2 (a)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1180,11 +1180,7 @@
           <t>DE 6.8.1 Parts 1-3</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Non-Newtonian Scientist due</t>
-        </is>
-      </c>
+      <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
@@ -1214,7 +1210,11 @@
           <t>6.166</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Non-Newtonian Scientist due</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Flex (freed when 2026-10-14 got a day ahead: a day ahead: Michael's two-day series plan put Taylor, the SymPy notebook and the crystal on Wed Oct 14 (class 14); Friday's content was covered (decided 2026-10-12 on the assumption that Wednesday lands))</t>
+          <t>Flex day</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Calendar: slip one meeting later after class 17 (matrix day taught Mon Oct 26 as class 19; Dec 14 flex day spent; Michael, 2026-10-26)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1167,19 +1167,15 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Determinants; finding eigenvalues and eigenvectors</t>
+          <t>Matrix multiplication; identity and inverse (continued)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>6.7-6.8</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>DE 6.8.1 Parts 1-3</t>
-        </is>
-      </c>
+          <t>6.5-6.6</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr"/>
       <c r="H23" s="2" t="inlineStr"/>
     </row>
@@ -1197,17 +1193,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Eigenvectors; the two-coupled-oscillator problem</t>
+          <t>Determinants; finding eigenvalues and eigenvectors</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>6.8-6.9</t>
+          <t>6.7-6.8</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>6.166</t>
+          <t>DE 6.8.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1231,17 +1227,17 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>Eigenvectors; the two-coupled-oscillator problem</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
+          <t>6.8-6.9</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.166</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1265,17 +1261,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals</t>
+          <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4</t>
+          <t>5.1-5.2</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>DE 5.4.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1295,15 +1291,19 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Polar coordinates</t>
+          <t>Cartesian 2D integrals</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5.6</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr"/>
+          <t>5.3-5.4</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.4.1</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
@@ -1321,19 +1321,15 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>Polar coordinates</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>5.163 parts a and d</t>
-        </is>
-      </c>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
@@ -1355,17 +1351,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Cylindrical and spherical coordinates</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>5.5, 5.7; App. D</t>
+          <t>5.8, 5.10</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>DE 5.7.1 Parts 1-4</t>
+          <t>5.163 parts a and d</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1385,17 +1381,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Vector and scalar fields; potential</t>
+          <t>Cylindrical and spherical coordinates</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>8.1-8.3</t>
+          <t>5.5, 5.7; App. D</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DE 8.2.1 Parts 5-6</t>
+          <t>DE 5.7.1 Parts 1-4</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1415,17 +1411,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>The gradient; equipotentials</t>
+          <t>Vector and scalar fields; potential</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.1-8.3</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>DE 8.4.1</t>
+          <t>DE 8.2.1 Parts 5-6</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1449,17 +1445,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Potential from a field; the gradient theorem; divergence and curl (Feynman)</t>
+          <t>The gradient; equipotentials</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>8.5-8.6; Feynman Vol II Ch 3</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Read Feynman II Ch 3 sections 3-1 to 3-6; in one or two sentences, what does the flux of a vector field out of a tiny box measure, and what does the circulation around a tiny loop measure?</t>
+          <t>DE 8.4.1</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -1479,17 +1475,17 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Divergence, curl, and the Laplacian; the divergence theorem</t>
+          <t>Potential from a field; the gradient theorem; divergence and curl (Feynman)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>8.6-8.7, 8.9; Feynman Vol II Ch 2</t>
+          <t>8.5-8.6; Feynman Vol II Ch 3</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>DE 8.6.1 Parts 1-9</t>
+          <t>Read Feynman II Ch 3 sections 3-1 to 3-6; in one or two sentences, what does the flux of a vector field out of a tiny box measure, and what does the circulation around a tiny loop measure?</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -1539,17 +1535,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Divergence theorem; Stokes' theorem</t>
+          <t>Divergence, curl, and the Laplacian; the divergence theorem</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>8.9-8.10</t>
+          <t>8.6-8.7, 8.9; Feynman Vol II Ch 2</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>DE 8.9.1</t>
+          <t>DE 8.6.1 Parts 1-9</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
@@ -1605,17 +1601,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Conservative vector fields</t>
+          <t>Divergence theorem; Stokes' theorem</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8.11</t>
+          <t>8.9-8.10</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
+          <t>DE 8.9.1</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -1635,17 +1631,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Introduction to Fourier series</t>
+          <t>Conservative vector fields</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>9.1-9.3</t>
+          <t>8.11</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>DE 9.2.1 Parts 1-3</t>
+          <t>DE 8.11.1 Parts 1-2, 4-5, 7-8</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
@@ -1665,17 +1661,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Fourier series: different periods, finite domains</t>
+          <t>Introduction to Fourier series</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.1-9.3</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>DE 9.4.1 Part 1</t>
+          <t>DE 9.2.1 Parts 1-3</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1699,15 +1695,19 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Fourier series with complex exponentials</t>
+          <t>Fourier series: different periods, finite domains</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>9.5</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>DE 9.4.1 Part 1</t>
+        </is>
+      </c>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr"/>
     </row>
@@ -1725,19 +1725,15 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Intro to PDEs: the heat equation; separation of variables</t>
+          <t>Fourier series with complex exponentials</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>11.1-11.2, 11.4</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>DE 11.2.1 Parts 1-2</t>
-        </is>
-      </c>
+          <t>9.5</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
     </row>
@@ -1755,17 +1751,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Normal modes of the wave equation; Fourier transforms</t>
+          <t>Intro to PDEs: the heat equation; separation of variables</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>11.3, 9.6</t>
+          <t>11.1-11.2, 11.4</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>DE 11.3.1 Part 1</t>
+          <t>DE 11.2.1 Parts 1-2</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -1789,11 +1785,19 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Flex day</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
+          <t>Normal modes of the wave equation; Fourier transforms</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>11.3, 9.6</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>DE 11.3.1 Part 1</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Calendar: class 21 (Oct 30) slipped a day; polar merged with cylindrical/spherical (Nov 9)
The equal-mass spring recap took the rest of class 21, so Mon Nov 2 (class 22) is a
continuation (springs spelled out, change of basis, carts capstone). Paid for inside
chapter 5, as Gary runs it: the polar day and the cylindrical/spherical day are one
"Polar, cylindrical and spherical coordinates" day (5.5-5.7; App. D), the freed slot is
a FLEX entry at Nov 11 consumed by the slip, and PCCI DE 5.7.1 Parts 1-4 follows its
topic. Chapter 8, the Nov 16 observed day and Quiz 3 do not move.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
+++ b/SyllabusAndFirstDay/2026/PHY210 F2026 Calendar.xlsx
@@ -1261,19 +1261,15 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Setting up 1D and 2D integrals</t>
+          <t>Eigenvectors; the two-coupled-oscillator problem (continued)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>5.1-5.2</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>5.1</t>
-        </is>
-      </c>
+          <t>6.8-6.9</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr"/>
     </row>
@@ -1291,17 +1287,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Cartesian 2D integrals</t>
+          <t>Setting up 1D and 2D integrals</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>5.3-5.4</t>
+          <t>5.1-5.2</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>DE 5.4.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1321,15 +1317,19 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Polar coordinates</t>
+          <t>Cartesian 2D integrals</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>5.6</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>5.3-5.4</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>DE 5.4.1</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>WHW09</t>
@@ -1351,17 +1351,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Line integrals and surface integrals</t>
+          <t>Polar, cylindrical and spherical coordinates</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>5.8, 5.10</t>
+          <t>5.5-5.7; App. D</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>5.163 parts a and d</t>
+          <t>DE 5.7.1 Parts 1-4</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1381,17 +1381,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Cylindrical and spherical coordinates</t>
+          <t>Line integrals and surface integrals</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>5.5, 5.7; App. D</t>
+          <t>5.8, 5.10</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DE 5.7.1 Parts 1-4</t>
+          <t>5.163 parts a and d</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>

</xml_diff>